<commit_message>
Add Type of Bill 327 tracking and email reporting
- Modified processPendingApproval to return both files and changedTo327 array
- Updated processPendingApprovalRecords to track all records changed to 327
- Modified processOffice to capture and pass through 327 changes
- Added 327 changes section to email body showing which records were changed
- Updated summary type to include changedTo327Count
- Added console logging for 327 changes per office
- Fixed early return in processPendingApprovalRecords to return empty array
</commit_message>
<xml_diff>
--- a/Insurance Instructions.xlsx
+++ b/Insurance Instructions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nightingale\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neerajvenu/ProjectSOLT/AI Projects/AI-BillingFromWellsky/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76C851DA-70A6-481A-9DA2-843884C57D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{341A29CD-2E83-DA4C-BB2D-DFCDE554FB64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{55CB68ED-2036-40CE-B779-4A0803795E7A}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="20740" windowHeight="11160" xr2:uid="{55CB68ED-2036-40CE-B779-4A0803795E7A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -697,11 +697,13 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color indexed="8"/>
-      <name val="verdana"/>
+      <name val="Verdana"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1135,14 +1137,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3C40B35-AD63-4714-8759-40B5CC9731DD}">
   <dimension ref="A1:C225"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.42578125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="91.1640625" customWidth="1"/>
+    <col min="3" max="3" width="53.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
@@ -1153,7 +1155,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1164,7 +1166,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1175,7 +1177,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -1186,7 +1188,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -1197,7 +1199,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1208,7 +1210,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -1219,7 +1221,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
@@ -1230,7 +1232,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -1241,7 +1243,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>5</v>
       </c>
@@ -1252,7 +1254,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
@@ -1263,7 +1265,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>5</v>
       </c>
@@ -1274,7 +1276,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>5</v>
       </c>
@@ -1285,7 +1287,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>5</v>
       </c>
@@ -1296,7 +1298,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
@@ -1307,7 +1309,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>5</v>
       </c>
@@ -1318,7 +1320,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>5</v>
       </c>
@@ -1329,7 +1331,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>5</v>
       </c>
@@ -1340,7 +1342,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>5</v>
       </c>
@@ -1351,7 +1353,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>5</v>
       </c>
@@ -1362,7 +1364,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>5</v>
       </c>
@@ -1373,7 +1375,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>5</v>
       </c>
@@ -1384,7 +1386,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>69</v>
       </c>
@@ -1395,7 +1397,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>69</v>
       </c>
@@ -1406,7 +1408,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>69</v>
       </c>
@@ -1417,7 +1419,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>69</v>
       </c>
@@ -1428,7 +1430,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>69</v>
       </c>
@@ -1439,7 +1441,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
@@ -1450,7 +1452,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>69</v>
       </c>
@@ -1461,7 +1463,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>69</v>
       </c>
@@ -1472,7 +1474,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>69</v>
       </c>
@@ -1483,7 +1485,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>69</v>
       </c>
@@ -1494,7 +1496,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>69</v>
       </c>
@@ -1505,7 +1507,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="77.25" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="71" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>69</v>
       </c>
@@ -1516,7 +1518,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>69</v>
       </c>
@@ -1527,7 +1529,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>69</v>
       </c>
@@ -1538,7 +1540,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>69</v>
       </c>
@@ -1549,7 +1551,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>69</v>
       </c>
@@ -1560,7 +1562,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>69</v>
       </c>
@@ -1571,7 +1573,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>69</v>
       </c>
@@ -1582,7 +1584,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>69</v>
       </c>
@@ -1593,7 +1595,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>69</v>
       </c>
@@ -1604,7 +1606,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>69</v>
       </c>
@@ -1615,7 +1617,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>69</v>
       </c>
@@ -1626,7 +1628,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
         <v>69</v>
       </c>
@@ -1637,7 +1639,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>69</v>
       </c>
@@ -1648,7 +1650,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
         <v>69</v>
       </c>
@@ -1659,7 +1661,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
         <v>69</v>
       </c>
@@ -1670,7 +1672,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>69</v>
       </c>
@@ -1681,7 +1683,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
         <v>69</v>
       </c>
@@ -1692,7 +1694,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>69</v>
       </c>
@@ -1703,7 +1705,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
         <v>69</v>
       </c>
@@ -1714,7 +1716,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>69</v>
       </c>
@@ -1725,7 +1727,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>69</v>
       </c>
@@ -1736,7 +1738,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>69</v>
       </c>
@@ -1747,7 +1749,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>69</v>
       </c>
@@ -1758,7 +1760,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
         <v>69</v>
       </c>
@@ -1769,7 +1771,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="39" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" ht="43" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
         <v>69</v>
       </c>
@@ -1780,7 +1782,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="39" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" ht="43" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
         <v>69</v>
       </c>
@@ -1791,7 +1793,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
         <v>69</v>
       </c>
@@ -1802,7 +1804,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>69</v>
       </c>
@@ -1813,7 +1815,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
         <v>69</v>
       </c>
@@ -1824,7 +1826,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>69</v>
       </c>
@@ -1835,7 +1837,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>69</v>
       </c>
@@ -1846,7 +1848,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>69</v>
       </c>
@@ -1857,7 +1859,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>69</v>
       </c>
@@ -1868,7 +1870,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>87</v>
       </c>
@@ -1879,7 +1881,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>87</v>
       </c>
@@ -1890,7 +1892,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>87</v>
       </c>
@@ -1901,7 +1903,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>87</v>
       </c>
@@ -1912,7 +1914,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>87</v>
       </c>
@@ -1923,7 +1925,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>87</v>
       </c>
@@ -1934,7 +1936,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>87</v>
       </c>
@@ -1945,7 +1947,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>87</v>
       </c>
@@ -1956,7 +1958,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>87</v>
       </c>
@@ -1967,7 +1969,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
         <v>87</v>
       </c>
@@ -1978,7 +1980,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
         <v>87</v>
       </c>
@@ -1989,7 +1991,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
         <v>87</v>
       </c>
@@ -2000,7 +2002,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>87</v>
       </c>
@@ -2011,7 +2013,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>87</v>
       </c>
@@ -2022,7 +2024,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
         <v>87</v>
       </c>
@@ -2033,7 +2035,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
         <v>87</v>
       </c>
@@ -2044,7 +2046,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>87</v>
       </c>
@@ -2055,7 +2057,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>87</v>
       </c>
@@ -2066,7 +2068,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>87</v>
       </c>
@@ -2077,7 +2079,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>87</v>
       </c>
@@ -2088,7 +2090,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>91</v>
       </c>
@@ -2099,7 +2101,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>91</v>
       </c>
@@ -2110,7 +2112,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>91</v>
       </c>
@@ -2121,7 +2123,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>104</v>
       </c>
@@ -2132,7 +2134,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
         <v>104</v>
       </c>
@@ -2143,7 +2145,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>104</v>
       </c>
@@ -2154,7 +2156,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>104</v>
       </c>
@@ -2165,7 +2167,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>104</v>
       </c>
@@ -2176,7 +2178,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>104</v>
       </c>
@@ -2187,7 +2189,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>104</v>
       </c>
@@ -2198,7 +2200,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>104</v>
       </c>
@@ -2209,7 +2211,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>104</v>
       </c>
@@ -2220,7 +2222,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>104</v>
       </c>
@@ -2231,7 +2233,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
         <v>104</v>
       </c>
@@ -2242,7 +2244,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
         <v>104</v>
       </c>
@@ -2253,7 +2255,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
         <v>104</v>
       </c>
@@ -2264,7 +2266,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
         <v>104</v>
       </c>
@@ -2275,7 +2277,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="7" t="s">
         <v>134</v>
       </c>
@@ -2286,7 +2288,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="7" t="s">
         <v>134</v>
       </c>
@@ -2297,7 +2299,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>134</v>
       </c>
@@ -2308,7 +2310,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" ht="57" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
         <v>134</v>
       </c>
@@ -2319,7 +2321,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
         <v>134</v>
       </c>
@@ -2330,7 +2332,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" s="7" t="s">
         <v>134</v>
       </c>
@@ -2341,7 +2343,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
         <v>134</v>
       </c>
@@ -2352,7 +2354,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="2" t="s">
         <v>134</v>
       </c>
@@ -2363,7 +2365,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
         <v>134</v>
       </c>
@@ -2374,7 +2376,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
         <v>134</v>
       </c>
@@ -2385,7 +2387,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="7" t="s">
         <v>134</v>
       </c>
@@ -2396,7 +2398,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
         <v>134</v>
       </c>
@@ -2407,7 +2409,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
         <v>134</v>
       </c>
@@ -2418,7 +2420,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
         <v>134</v>
       </c>
@@ -2429,7 +2431,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
         <v>134</v>
       </c>
@@ -2440,7 +2442,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
         <v>134</v>
       </c>
@@ -2451,7 +2453,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
         <v>134</v>
       </c>
@@ -2462,7 +2464,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" s="2" t="s">
         <v>134</v>
       </c>
@@ -2473,7 +2475,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" s="2" t="s">
         <v>134</v>
       </c>
@@ -2484,7 +2486,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" s="7" t="s">
         <v>134</v>
       </c>
@@ -2495,7 +2497,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" s="7" t="s">
         <v>134</v>
       </c>
@@ -2506,7 +2508,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A125" s="7" t="s">
         <v>134</v>
       </c>
@@ -2517,7 +2519,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A126" s="2" t="s">
         <v>134</v>
       </c>
@@ -2528,7 +2530,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A127" s="2" t="s">
         <v>134</v>
       </c>
@@ -2539,7 +2541,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" ht="71" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
         <v>134</v>
       </c>
@@ -2550,7 +2552,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" s="2" t="s">
         <v>134</v>
       </c>
@@ -2561,7 +2563,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" s="2" t="s">
         <v>134</v>
       </c>
@@ -2572,7 +2574,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" s="2" t="s">
         <v>134</v>
       </c>
@@ -2583,7 +2585,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="132" spans="1:3" ht="102.75" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" ht="99" x14ac:dyDescent="0.2">
       <c r="A132" s="4" t="s">
         <v>134</v>
       </c>
@@ -2594,7 +2596,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" s="2" t="s">
         <v>134</v>
       </c>
@@ -2605,7 +2607,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" s="2" t="s">
         <v>3</v>
       </c>
@@ -2616,7 +2618,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A135" s="2" t="s">
         <v>3</v>
       </c>
@@ -2627,7 +2629,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A136" s="2" t="s">
         <v>3</v>
       </c>
@@ -2638,7 +2640,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
         <v>3</v>
       </c>
@@ -2649,7 +2651,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A138" s="2" t="s">
         <v>3</v>
       </c>
@@ -2660,7 +2662,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A139" s="2" t="s">
         <v>3</v>
       </c>
@@ -2671,7 +2673,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A140" s="2" t="s">
         <v>3</v>
       </c>
@@ -2682,7 +2684,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
         <v>3</v>
       </c>
@@ -2693,7 +2695,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
         <v>3</v>
       </c>
@@ -2704,7 +2706,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A143" s="2" t="s">
         <v>3</v>
       </c>
@@ -2715,7 +2717,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A144" s="2" t="s">
         <v>3</v>
       </c>
@@ -2726,7 +2728,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A145" s="2" t="s">
         <v>3</v>
       </c>
@@ -2737,7 +2739,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A146" s="2" t="s">
         <v>3</v>
       </c>
@@ -2748,7 +2750,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A147" s="2" t="s">
         <v>3</v>
       </c>
@@ -2759,7 +2761,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A148" s="2" t="s">
         <v>3</v>
       </c>
@@ -2770,7 +2772,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A149" s="2" t="s">
         <v>3</v>
       </c>
@@ -2781,7 +2783,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A150" s="2" t="s">
         <v>3</v>
       </c>
@@ -2792,7 +2794,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A151" s="2" t="s">
         <v>158</v>
       </c>
@@ -2803,7 +2805,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A152" s="2" t="s">
         <v>158</v>
       </c>
@@ -2814,7 +2816,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A153" s="2" t="s">
         <v>158</v>
       </c>
@@ -2825,7 +2827,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A154" s="2" t="s">
         <v>158</v>
       </c>
@@ -2836,7 +2838,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A155" s="2" t="s">
         <v>158</v>
       </c>
@@ -2847,7 +2849,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A156" s="2" t="s">
         <v>158</v>
       </c>
@@ -2858,7 +2860,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A157" s="2" t="s">
         <v>158</v>
       </c>
@@ -2869,7 +2871,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" s="2" t="s">
         <v>158</v>
       </c>
@@ -2880,7 +2882,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" s="2" t="s">
         <v>158</v>
       </c>
@@ -2891,7 +2893,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
         <v>158</v>
       </c>
@@ -2902,7 +2904,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
         <v>158</v>
       </c>
@@ -2913,7 +2915,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A162" s="2" t="s">
         <v>158</v>
       </c>
@@ -2924,7 +2926,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A163" s="2" t="s">
         <v>158</v>
       </c>
@@ -2935,7 +2937,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A164" s="2" t="s">
         <v>158</v>
       </c>
@@ -2946,7 +2948,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A165" s="2" t="s">
         <v>158</v>
       </c>
@@ -2957,7 +2959,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A166" s="2" t="s">
         <v>170</v>
       </c>
@@ -2968,7 +2970,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A167" s="2" t="s">
         <v>170</v>
       </c>
@@ -2979,7 +2981,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A168" s="2" t="s">
         <v>170</v>
       </c>
@@ -2990,7 +2992,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A169" s="2" t="s">
         <v>170</v>
       </c>
@@ -3001,7 +3003,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A170" s="2" t="s">
         <v>170</v>
       </c>
@@ -3012,7 +3014,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A171" s="2" t="s">
         <v>170</v>
       </c>
@@ -3023,7 +3025,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A172" s="2" t="s">
         <v>170</v>
       </c>
@@ -3034,7 +3036,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A173" s="2" t="s">
         <v>170</v>
       </c>
@@ -3045,7 +3047,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A174" s="2" t="s">
         <v>170</v>
       </c>
@@ -3056,7 +3058,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A175" s="4" t="s">
         <v>170</v>
       </c>
@@ -3067,7 +3069,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A176" s="2" t="s">
         <v>170</v>
       </c>
@@ -3078,7 +3080,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A177" s="2" t="s">
         <v>208</v>
       </c>
@@ -3089,7 +3091,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A178" s="2" t="s">
         <v>208</v>
       </c>
@@ -3100,7 +3102,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A179" s="2" t="s">
         <v>208</v>
       </c>
@@ -3111,7 +3113,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A180" s="2" t="s">
         <v>208</v>
       </c>
@@ -3122,7 +3124,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A181" s="2" t="s">
         <v>208</v>
       </c>
@@ -3133,7 +3135,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A182" s="2" t="s">
         <v>208</v>
       </c>
@@ -3144,7 +3146,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A183" s="2" t="s">
         <v>208</v>
       </c>
@@ -3155,7 +3157,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A184" s="2" t="s">
         <v>208</v>
       </c>
@@ -3166,7 +3168,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A185" s="2" t="s">
         <v>208</v>
       </c>
@@ -3177,7 +3179,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A186" s="2" t="s">
         <v>208</v>
       </c>
@@ -3188,7 +3190,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A187" s="2" t="s">
         <v>208</v>
       </c>
@@ -3199,7 +3201,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A188" s="2" t="s">
         <v>208</v>
       </c>
@@ -3210,7 +3212,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A189" s="7" t="s">
         <v>208</v>
       </c>
@@ -3221,7 +3223,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A190" s="2" t="s">
         <v>208</v>
       </c>
@@ -3232,7 +3234,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A191" s="2" t="s">
         <v>208</v>
       </c>
@@ -3243,7 +3245,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A192" s="2" t="s">
         <v>208</v>
       </c>
@@ -3254,7 +3256,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A193" s="2" t="s">
         <v>208</v>
       </c>
@@ -3265,7 +3267,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A194" s="2" t="s">
         <v>208</v>
       </c>
@@ -3276,7 +3278,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A195" s="2" t="s">
         <v>208</v>
       </c>
@@ -3287,7 +3289,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A196" s="2" t="s">
         <v>208</v>
       </c>
@@ -3298,7 +3300,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A197" s="2" t="s">
         <v>208</v>
       </c>
@@ -3309,7 +3311,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A198" s="2" t="s">
         <v>208</v>
       </c>
@@ -3320,7 +3322,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A199" s="2" t="s">
         <v>208</v>
       </c>
@@ -3331,7 +3333,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A200" s="2" t="s">
         <v>208</v>
       </c>
@@ -3342,7 +3344,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A201" s="2" t="s">
         <v>208</v>
       </c>
@@ -3353,7 +3355,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A202" s="2" t="s">
         <v>208</v>
       </c>
@@ -3364,7 +3366,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A203" s="2" t="s">
         <v>208</v>
       </c>
@@ -3375,7 +3377,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A204" s="2" t="s">
         <v>208</v>
       </c>
@@ -3386,7 +3388,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A205" s="2" t="s">
         <v>208</v>
       </c>
@@ -3397,7 +3399,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A206" s="2" t="s">
         <v>208</v>
       </c>
@@ -3408,7 +3410,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A207" s="2" t="s">
         <v>208</v>
       </c>
@@ -3419,7 +3421,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A208" s="2" t="s">
         <v>208</v>
       </c>
@@ -3430,7 +3432,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A209" s="2" t="s">
         <v>208</v>
       </c>
@@ -3441,7 +3443,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A210" s="2" t="s">
         <v>208</v>
       </c>
@@ -3452,7 +3454,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A211" s="2" t="s">
         <v>208</v>
       </c>
@@ -3463,7 +3465,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A212" s="7" t="s">
         <v>208</v>
       </c>
@@ -3474,7 +3476,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A213" s="2" t="s">
         <v>208</v>
       </c>
@@ -3485,7 +3487,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A214" s="7" t="s">
         <v>208</v>
       </c>
@@ -3496,7 +3498,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A215" s="7" t="s">
         <v>208</v>
       </c>
@@ -3507,7 +3509,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A216" s="4" t="s">
         <v>208</v>
       </c>
@@ -3518,7 +3520,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A217" s="2" t="s">
         <v>208</v>
       </c>
@@ -3529,7 +3531,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A218" s="2" t="s">
         <v>208</v>
       </c>
@@ -3540,7 +3542,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A219" s="2" t="s">
         <v>208</v>
       </c>
@@ -3551,7 +3553,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A220" s="7" t="s">
         <v>208</v>
       </c>
@@ -3562,7 +3564,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A221" s="7" t="s">
         <v>208</v>
       </c>
@@ -3573,7 +3575,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A222" s="7" t="s">
         <v>208</v>
       </c>
@@ -3584,7 +3586,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A223" s="2" t="s">
         <v>208</v>
       </c>
@@ -3595,7 +3597,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A224" s="2" t="s">
         <v>208</v>
       </c>
@@ -3606,7 +3608,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A225" s="2" t="s">
         <v>208</v>
       </c>

</xml_diff>

<commit_message>
Update Insurance Instructions.xlsx - fix FALLON COMMUNITY HEALTH PLAN MAV spelling
</commit_message>
<xml_diff>
--- a/Insurance Instructions.xlsx
+++ b/Insurance Instructions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neerajvenu/ProjectSOLT/AI Projects/AI-BillingFromWellsky/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E02ADAF-94EE-A24C-9D0A-0FCB6DE48057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF82E0BD-E419-6F41-BEB2-EE5CE484A93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20740" windowHeight="11160" xr2:uid="{55CB68ED-2036-40CE-B779-4A0803795E7A}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{55CB68ED-2036-40CE-B779-4A0803795E7A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -393,9 +393,6 @@
     <t>Eternal Health</t>
   </si>
   <si>
-    <t>FALLON COMMNITY HEALTH PLAN MAV</t>
-  </si>
-  <si>
     <t>Need to check for G code and T code from Authorizations. And also if there is any patient where two SN visits are being done same day. Need to make sure both SN visits are there in the claim form.</t>
   </si>
   <si>
@@ -680,6 +677,9 @@
   </si>
   <si>
     <t>No changes are required except for identical claims.</t>
+  </si>
+  <si>
+    <t>FALLON COMMUNITY HEALTH PLAN MAV</t>
   </si>
 </sst>
 </file>
@@ -1152,7 +1152,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1163,7 +1163,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -1174,7 +1174,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1185,7 +1185,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -1196,7 +1196,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1207,7 +1207,7 @@
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1218,7 +1218,7 @@
         <v>9</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -1229,7 +1229,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -1240,7 +1240,7 @@
         <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -1251,7 +1251,7 @@
         <v>12</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -1262,7 +1262,7 @@
         <v>13</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -1273,7 +1273,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -1284,7 +1284,7 @@
         <v>15</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -1295,7 +1295,7 @@
         <v>16</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -1306,7 +1306,7 @@
         <v>17</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -1317,7 +1317,7 @@
         <v>18</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -1328,7 +1328,7 @@
         <v>19</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -1339,7 +1339,7 @@
         <v>20</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -1350,7 +1350,7 @@
         <v>21</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -1361,7 +1361,7 @@
         <v>22</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -1372,7 +1372,7 @@
         <v>23</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -1383,7 +1383,7 @@
         <v>24</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
@@ -1394,7 +1394,7 @@
         <v>26</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -1405,7 +1405,7 @@
         <v>27</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -1416,7 +1416,7 @@
         <v>28</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -1427,7 +1427,7 @@
         <v>29</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -1438,7 +1438,7 @@
         <v>30</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -1449,7 +1449,7 @@
         <v>31</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -1460,7 +1460,7 @@
         <v>32</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -1471,7 +1471,7 @@
         <v>33</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -1482,7 +1482,7 @@
         <v>34</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -1493,7 +1493,7 @@
         <v>35</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -1504,7 +1504,7 @@
         <v>9</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="71" x14ac:dyDescent="0.2">
@@ -1526,7 +1526,7 @@
         <v>38</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
@@ -1537,7 +1537,7 @@
         <v>12</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
@@ -1548,7 +1548,7 @@
         <v>39</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -1559,7 +1559,7 @@
         <v>40</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
@@ -1570,7 +1570,7 @@
         <v>13</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
@@ -1581,7 +1581,7 @@
         <v>41</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
@@ -1592,7 +1592,7 @@
         <v>42</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -1603,7 +1603,7 @@
         <v>43</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
@@ -1614,7 +1614,7 @@
         <v>44</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
@@ -1625,7 +1625,7 @@
         <v>45</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
@@ -1647,7 +1647,7 @@
         <v>15</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -1680,7 +1680,7 @@
         <v>50</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -1691,7 +1691,7 @@
         <v>51</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
@@ -1702,7 +1702,7 @@
         <v>52</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
@@ -1713,7 +1713,7 @@
         <v>53</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -1724,7 +1724,7 @@
         <v>54</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -1735,7 +1735,7 @@
         <v>55</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -1746,7 +1746,7 @@
         <v>56</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
@@ -1757,7 +1757,7 @@
         <v>57</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -1834,7 +1834,7 @@
         <v>22</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
@@ -1845,7 +1845,7 @@
         <v>66</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
@@ -1856,7 +1856,7 @@
         <v>67</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
@@ -1867,7 +1867,7 @@
         <v>68</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
@@ -1878,7 +1878,7 @@
         <v>26</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
@@ -1889,7 +1889,7 @@
         <v>70</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -1900,7 +1900,7 @@
         <v>71</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
@@ -1911,7 +1911,7 @@
         <v>72</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -1922,7 +1922,7 @@
         <v>73</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
@@ -1933,7 +1933,7 @@
         <v>74</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
@@ -1944,7 +1944,7 @@
         <v>75</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -1955,7 +1955,7 @@
         <v>38</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -1966,7 +1966,7 @@
         <v>76</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -2010,7 +2010,7 @@
         <v>79</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
@@ -2021,7 +2021,7 @@
         <v>80</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -2054,7 +2054,7 @@
         <v>83</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
@@ -2065,7 +2065,7 @@
         <v>84</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
@@ -2076,7 +2076,7 @@
         <v>85</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
@@ -2087,7 +2087,7 @@
         <v>86</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -2098,7 +2098,7 @@
         <v>88</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -2109,7 +2109,7 @@
         <v>89</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -2120,7 +2120,7 @@
         <v>90</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -2131,7 +2131,7 @@
         <v>92</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -2153,7 +2153,7 @@
         <v>94</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
@@ -2164,7 +2164,7 @@
         <v>95</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -2175,7 +2175,7 @@
         <v>96</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
@@ -2186,7 +2186,7 @@
         <v>13</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -2197,7 +2197,7 @@
         <v>97</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -2208,7 +2208,7 @@
         <v>98</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -2219,7 +2219,7 @@
         <v>99</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
@@ -2230,7 +2230,7 @@
         <v>100</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
@@ -2241,7 +2241,7 @@
         <v>80</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -2252,7 +2252,7 @@
         <v>101</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
@@ -2263,7 +2263,7 @@
         <v>102</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
@@ -2274,12 +2274,12 @@
         <v>103</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B104" s="8" t="s">
         <v>105</v>
@@ -2290,7 +2290,7 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B105" s="8" t="s">
         <v>106</v>
@@ -2301,18 +2301,18 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="107" spans="1:3" ht="57" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>107</v>
@@ -2323,18 +2323,18 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>109</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B109" s="8" t="s">
         <v>110</v>
@@ -2345,40 +2345,40 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B110" s="3" t="s">
         <v>111</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B111" s="3" t="s">
         <v>112</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B112" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>113</v>
@@ -2389,7 +2389,7 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B114" s="8" t="s">
         <v>115</v>
@@ -2400,95 +2400,95 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B115" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="C115" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="C115" s="10" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B120" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B123" s="8" t="s">
         <v>46</v>
@@ -2499,10 +2499,10 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B124" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C124" s="8" t="s">
         <v>47</v>
@@ -2510,10 +2510,10 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A125" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C125" s="8" t="s">
         <v>47</v>
@@ -2521,90 +2521,90 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A126" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B126" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A127" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="71" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B128" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C128" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="C128" s="6" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="132" spans="1:3" ht="99" x14ac:dyDescent="0.2">
       <c r="A132" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B132" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C132" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="C132" s="6" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
@@ -2612,10 +2612,10 @@
         <v>3</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
@@ -2623,10 +2623,10 @@
         <v>3</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
@@ -2637,7 +2637,7 @@
         <v>75</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
@@ -2645,10 +2645,10 @@
         <v>3</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
@@ -2656,10 +2656,10 @@
         <v>3</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
@@ -2667,10 +2667,10 @@
         <v>3</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
@@ -2678,10 +2678,10 @@
         <v>3</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
@@ -2689,10 +2689,10 @@
         <v>3</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
@@ -2703,7 +2703,7 @@
         <v>13</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
@@ -2711,10 +2711,10 @@
         <v>3</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
@@ -2722,10 +2722,10 @@
         <v>3</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
@@ -2736,7 +2736,7 @@
         <v>80</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
@@ -2744,10 +2744,10 @@
         <v>3</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.2">
@@ -2755,10 +2755,10 @@
         <v>3</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
@@ -2766,10 +2766,10 @@
         <v>3</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
@@ -2777,10 +2777,10 @@
         <v>3</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
@@ -2788,436 +2788,436 @@
         <v>3</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A151" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A152" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A153" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A154" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A155" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A156" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A157" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B158" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A162" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B162" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A163" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A164" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A165" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A166" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A167" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B167" s="3" t="s">
         <v>71</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A168" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A169" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B169" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A170" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A171" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A172" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A173" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A174" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A175" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B175" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C175" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="C175" s="5" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A176" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A177" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A178" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C178" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A179" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A180" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C180" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A181" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A182" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>30</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A183" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A184" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A185" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A186" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>110</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A187" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A188" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A189" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B189" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C189" s="8" t="s">
         <v>47</v>
@@ -3225,252 +3225,252 @@
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A190" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A191" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B191" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A192" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A193" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A194" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A195" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C195" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A196" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C196" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A197" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C197" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A198" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C198" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A199" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A200" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B200" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C200" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A201" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C201" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A202" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B202" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A203" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A204" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A205" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A206" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B206" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A207" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A208" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A209" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A210" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A211" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A212" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B212" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C212" s="8" t="s">
         <v>47</v>
@@ -3478,18 +3478,18 @@
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A213" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B213" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A214" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B214" s="8" t="s">
         <v>17</v>
@@ -3500,7 +3500,7 @@
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A215" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B215" s="8" t="s">
         <v>49</v>
@@ -3511,112 +3511,112 @@
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A216" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B216" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="C216" s="5" t="s">
         <v>197</v>
-      </c>
-      <c r="C216" s="5" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A217" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C217" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A218" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B218" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A219" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B219" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C219" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A220" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B220" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C220" s="8" t="s">
         <v>201</v>
-      </c>
-      <c r="C220" s="8" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A221" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B221" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C221" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A222" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B222" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C222" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A223" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B223" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A224" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C224" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A225" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B225" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C225" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Northcoast -Aetna and Northcost PPS- Anthem to spreadsheet and code (OH office, exact names from Kinnser)
</commit_message>
<xml_diff>
--- a/Insurance Instructions.xlsx
+++ b/Insurance Instructions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neerajvenu/ProjectSOLT/AI Projects/AI-BillingFromWellsky/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF82E0BD-E419-6F41-BEB2-EE5CE484A93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DFE19F0-A853-AD46-B65E-68AFE7F214F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{55CB68ED-2036-40CE-B779-4A0803795E7A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$225</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$226</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="212">
   <si>
     <t>Name</t>
   </si>
@@ -680,6 +680,9 @@
   </si>
   <si>
     <t>FALLON COMMUNITY HEALTH PLAN MAV</t>
+  </si>
+  <si>
+    <t>Northcoast -Aetna</t>
   </si>
 </sst>
 </file>
@@ -1136,7 +1139,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3C40B35-AD63-4714-8759-40B5CC9731DD}">
-  <dimension ref="A1:C225"/>
+  <dimension ref="A1:C226"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" bestFit="1" customWidth="1"/>
@@ -3059,33 +3062,33 @@
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A175" s="4" t="s">
+      <c r="A175" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B175" s="5" t="s">
-        <v>166</v>
+      <c r="B175" s="3" t="s">
+        <v>211</v>
       </c>
       <c r="C175" s="5" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A176" s="2" t="s">
+      <c r="A176" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B176" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="C176" s="3" t="s">
-        <v>209</v>
+      <c r="B176" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C176" s="5" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A177" s="2" t="s">
-        <v>207</v>
+        <v>169</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C177" s="3" t="s">
         <v>209</v>
@@ -3096,7 +3099,7 @@
         <v>207</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C178" s="3" t="s">
         <v>209</v>
@@ -3107,7 +3110,7 @@
         <v>207</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C179" s="3" t="s">
         <v>209</v>
@@ -3118,7 +3121,7 @@
         <v>207</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C180" s="3" t="s">
         <v>209</v>
@@ -3129,7 +3132,7 @@
         <v>207</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>8</v>
+        <v>173</v>
       </c>
       <c r="C181" s="3" t="s">
         <v>209</v>
@@ -3140,7 +3143,7 @@
         <v>207</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C182" s="3" t="s">
         <v>209</v>
@@ -3151,7 +3154,7 @@
         <v>207</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C183" s="3" t="s">
         <v>209</v>
@@ -3162,7 +3165,7 @@
         <v>207</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>174</v>
+        <v>31</v>
       </c>
       <c r="C184" s="3" t="s">
         <v>209</v>
@@ -3173,7 +3176,7 @@
         <v>207</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C185" s="3" t="s">
         <v>209</v>
@@ -3184,7 +3187,7 @@
         <v>207</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>110</v>
+        <v>175</v>
       </c>
       <c r="C186" s="3" t="s">
         <v>209</v>
@@ -3195,7 +3198,7 @@
         <v>207</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>176</v>
+        <v>110</v>
       </c>
       <c r="C187" s="3" t="s">
         <v>209</v>
@@ -3206,32 +3209,32 @@
         <v>207</v>
       </c>
       <c r="B188" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C188" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A189" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B189" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C188" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A189" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="B189" s="8" t="s">
+      <c r="C189" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A190" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B190" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="C189" s="8" t="s">
+      <c r="C190" s="8" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A190" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="B190" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C190" s="3" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.2">
@@ -3239,7 +3242,7 @@
         <v>207</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>9</v>
+        <v>179</v>
       </c>
       <c r="C191" s="3" t="s">
         <v>209</v>
@@ -3250,7 +3253,7 @@
         <v>207</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>180</v>
+        <v>9</v>
       </c>
       <c r="C192" s="3" t="s">
         <v>209</v>
@@ -3261,7 +3264,7 @@
         <v>207</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C193" s="3" t="s">
         <v>209</v>
@@ -3272,7 +3275,7 @@
         <v>207</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C194" s="3" t="s">
         <v>209</v>
@@ -3283,7 +3286,7 @@
         <v>207</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C195" s="3" t="s">
         <v>209</v>
@@ -3294,7 +3297,7 @@
         <v>207</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C196" s="3" t="s">
         <v>209</v>
@@ -3305,7 +3308,7 @@
         <v>207</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C197" s="3" t="s">
         <v>209</v>
@@ -3316,7 +3319,7 @@
         <v>207</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>119</v>
+        <v>185</v>
       </c>
       <c r="C198" s="3" t="s">
         <v>209</v>
@@ -3327,7 +3330,7 @@
         <v>207</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>186</v>
+        <v>119</v>
       </c>
       <c r="C199" s="3" t="s">
         <v>209</v>
@@ -3338,7 +3341,7 @@
         <v>207</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>40</v>
+        <v>186</v>
       </c>
       <c r="C200" s="3" t="s">
         <v>209</v>
@@ -3349,7 +3352,7 @@
         <v>207</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>187</v>
+        <v>40</v>
       </c>
       <c r="C201" s="3" t="s">
         <v>209</v>
@@ -3360,7 +3363,7 @@
         <v>207</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>41</v>
+        <v>187</v>
       </c>
       <c r="C202" s="3" t="s">
         <v>209</v>
@@ -3371,7 +3374,7 @@
         <v>207</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>188</v>
+        <v>41</v>
       </c>
       <c r="C203" s="3" t="s">
         <v>209</v>
@@ -3382,7 +3385,7 @@
         <v>207</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C204" s="3" t="s">
         <v>209</v>
@@ -3393,7 +3396,7 @@
         <v>207</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C205" s="3" t="s">
         <v>209</v>
@@ -3404,7 +3407,7 @@
         <v>207</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>43</v>
+        <v>190</v>
       </c>
       <c r="C206" s="3" t="s">
         <v>209</v>
@@ -3415,7 +3418,7 @@
         <v>207</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>191</v>
+        <v>43</v>
       </c>
       <c r="C207" s="3" t="s">
         <v>209</v>
@@ -3426,7 +3429,7 @@
         <v>207</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C208" s="3" t="s">
         <v>209</v>
@@ -3437,7 +3440,7 @@
         <v>207</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C209" s="3" t="s">
         <v>209</v>
@@ -3448,7 +3451,7 @@
         <v>207</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C210" s="3" t="s">
         <v>209</v>
@@ -3459,43 +3462,43 @@
         <v>207</v>
       </c>
       <c r="B211" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="C211" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A212" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B212" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C211" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A212" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="B212" s="8" t="s">
+      <c r="C212" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A213" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B213" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="C212" s="8" t="s">
+      <c r="C213" s="8" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A213" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="B213" s="3" t="s">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A214" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B214" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C213" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A214" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="B214" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C214" s="8" t="s">
-        <v>47</v>
+      <c r="C214" s="3" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.2">
@@ -3503,32 +3506,32 @@
         <v>207</v>
       </c>
       <c r="B215" s="8" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C215" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A216" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="B216" s="5" t="s">
+      <c r="A216" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B216" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C216" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A217" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B217" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="C216" s="5" t="s">
+      <c r="C217" s="5" t="s">
         <v>197</v>
-      </c>
-    </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A217" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="B217" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C217" s="3" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.2">
@@ -3536,7 +3539,7 @@
         <v>207</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>80</v>
+        <v>198</v>
       </c>
       <c r="C218" s="3" t="s">
         <v>209</v>
@@ -3547,21 +3550,21 @@
         <v>207</v>
       </c>
       <c r="B219" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C219" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A220" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B220" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="C219" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A220" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="B220" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="C220" s="8" t="s">
-        <v>201</v>
+      <c r="C220" s="3" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.2">
@@ -3569,7 +3572,7 @@
         <v>207</v>
       </c>
       <c r="B221" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C221" s="8" t="s">
         <v>201</v>
@@ -3580,21 +3583,21 @@
         <v>207</v>
       </c>
       <c r="B222" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C222" s="8" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A223" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="B223" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="C223" s="3" t="s">
-        <v>209</v>
+      <c r="A223" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B223" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="C223" s="8" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.2">
@@ -3602,7 +3605,7 @@
         <v>207</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C224" s="3" t="s">
         <v>209</v>
@@ -3613,9 +3616,20 @@
         <v>207</v>
       </c>
       <c r="B225" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A226" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B226" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="C225" s="3" t="s">
+      <c r="C226" s="3" t="s">
         <v>209</v>
       </c>
     </row>

</xml_diff>